<commit_message>
Upload Excel file CV Discount Check Master File 08.05.2026.xlsx
</commit_message>
<xml_diff>
--- a/Data/Discount_Cheker/CV Discount Check Master File 08.05.2026.xlsx
+++ b/Data/Discount_Cheker/CV Discount Check Master File 08.05.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Auditor RSM Data\To be Consider\2026-27\2. May-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5CC4F87-000E-4427-991F-A35D1D4F3083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CEF10BD-2D30-42DA-98BE-7E206E87450C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{9C2300AC-C402-454B-B7CF-00A24C218261}"/>
   </bookViews>
@@ -429,7 +429,7 @@
     <t>21K + RSA FREE</t>
   </si>
   <si>
-    <t>MAY-2026 (VIN 2026)</t>
+    <t>MAY-2026 - VIN 2026</t>
   </si>
 </sst>
 </file>
@@ -5183,21 +5183,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010060EDED336F4AC345937821C4378B0575" ma:contentTypeVersion="13" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="494f29b6abfd1a658fb4a91257319fb7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="cc81ea25-3c65-47fe-b799-37236d34457b" xmlns:ns4="3aa501bf-b653-40a4-9ae9-61a4d1229c70" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="79a9a6d6e67940bfc0c15f927b8771f4" ns3:_="" ns4:_="">
     <xsd:import namespace="cc81ea25-3c65-47fe-b799-37236d34457b"/>
@@ -5420,24 +5405,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9062C800-B5CF-4467-9EC7-2088426858BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{250AA7BD-7B6E-43C6-AED0-1E579093AA92}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6B08E05-D3E6-4391-8AA6-C9B1EA9A23D0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5454,4 +5437,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{250AA7BD-7B6E-43C6-AED0-1E579093AA92}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9062C800-B5CF-4467-9EC7-2088426858BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>